<commit_message>
add: test examples data and voice
</commit_message>
<xml_diff>
--- a/Mapping/test_case_map.xlsx
+++ b/Mapping/test_case_map.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daffaarifadilah/techbros/fInal_parsing/Mapping/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daffaarifadilah/techbros/fInal_parsing/Code/Mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F366D6-0B2E-8949-8DDB-B15FDC54D233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46915D12-5055-C14C-A1E4-FD6098EE0362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{1E68A79A-A9F1-49C0-BB8D-402639C0A121}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="24000" xr2:uid="{1E68A79A-A9F1-49C0-BB8D-402639C0A121}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="88">
   <si>
     <t>Test Name</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>URI: http://uploadtest.techbros.io/upload-fdtt</t>
+  </si>
+  <si>
+    <t>Source Uri: https://www.youtube.com/watch?v=bNyUyrR0PHo</t>
   </si>
 </sst>
 </file>
@@ -465,7 +468,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -528,6 +531,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -886,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC2CE570-82D3-4CA5-B308-9D4F3DEBB424}">
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="85" style="14" bestFit="1" customWidth="1"/>
@@ -1775,7 +1781,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="17" t="s">
         <v>38</v>
       </c>
@@ -1786,7 +1792,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="17" t="s">
         <v>59</v>
       </c>
@@ -1797,7 +1803,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="17" t="s">
         <v>43</v>
       </c>
@@ -1808,7 +1814,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="17" t="s">
         <v>44</v>
       </c>
@@ -1819,7 +1825,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="15" t="s">
         <v>46</v>
       </c>
@@ -1829,9 +1835,8 @@
       <c r="C85" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D85" s="21"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="15" t="s">
         <v>47</v>
       </c>
@@ -1841,9 +1846,8 @@
       <c r="C86" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D86" s="21"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>81</v>
       </c>
@@ -1853,9 +1857,8 @@
       <c r="C87" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D87" s="21"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>82</v>
       </c>
@@ -1865,9 +1868,8 @@
       <c r="C88" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D88" s="21"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -1877,9 +1879,8 @@
       <c r="C89" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D89" s="21"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>84</v>
       </c>
@@ -1889,9 +1890,8 @@
       <c r="C90" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D90" s="21"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>85</v>
       </c>
@@ -1901,9 +1901,8 @@
       <c r="C91" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D91" s="21"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="17" t="s">
         <v>53</v>
       </c>
@@ -1914,7 +1913,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="17" t="s">
         <v>54</v>
       </c>
@@ -1925,7 +1924,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="17" t="s">
         <v>55</v>
       </c>
@@ -1936,7 +1935,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="17" t="s">
         <v>56</v>
       </c>
@@ -1947,7 +1946,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="17" t="s">
         <v>57</v>
       </c>
@@ -2001,6 +2000,42 @@
       <c r="C100" s="25" t="s">
         <v>77</v>
       </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B101" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C101" s="25" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B102" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C102" s="25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B103" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C103" s="25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104" s="26"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A64:A76">
@@ -2025,5 +2060,6 @@
     <hyperlink ref="A39" r:id="rId13" display="https://www.youtube.com/watch?v=BQwC_DJSdfE" xr:uid="{0F9953AD-223E-4DB0-B12E-8F6F461F062A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>